<commit_message>
Update assignment and pacing
</commit_message>
<xml_diff>
--- a/Pacing_Dates_Master.xlsx
+++ b/Pacing_Dates_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\GCI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A4655B58-D611-4107-868E-04DB1A558A19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF452411-42C2-4979-AF9B-298592F22B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{327FF7BE-3859-42FE-861D-17B3CC93C4A1}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1187" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="126">
   <si>
     <t>SourceType</t>
   </si>
@@ -324,9 +324,6 @@
     <t>PCEP Certification</t>
   </si>
   <si>
-    <t>Design Thinking</t>
-  </si>
-  <si>
     <t>Virtual Assignment</t>
   </si>
   <si>
@@ -348,38 +345,75 @@
     <t>All hardware classes</t>
   </si>
   <si>
-    <t>All hardware classes (2nd session)</t>
-  </si>
-  <si>
     <t>AP Computer Science A: Game Design</t>
   </si>
   <si>
-    <t>3rd session AP Computer Science A</t>
-  </si>
-  <si>
-    <t>Website Checkpoint 1</t>
-  </si>
-  <si>
     <t>AP Computer Science A milestone</t>
   </si>
   <si>
     <t>AP Computer Science A final website due</t>
   </si>
   <si>
-    <t>Website Checkpoint 2</t>
-  </si>
-  <si>
     <t>AP Exam</t>
   </si>
   <si>
     <t>Deadline for submissions for MP3</t>
+  </si>
+  <si>
+    <t>IT Specialist Certification - Python Practice Test</t>
+  </si>
+  <si>
+    <t>Three Keys - QA Project</t>
+  </si>
+  <si>
+    <t>5.4: Forensic Case 3: Exif Data</t>
+  </si>
+  <si>
+    <t>Catch up/Brain Break</t>
+  </si>
+  <si>
+    <t>Teamwork Assignment Due - Catch up/Brain Break</t>
+  </si>
+  <si>
+    <t>9.1: Identifying Risks</t>
+  </si>
+  <si>
+    <t>9.2: Assessing Risks</t>
+  </si>
+  <si>
+    <t>9.3: Risk Response</t>
+  </si>
+  <si>
+    <t>9.4: Penetration Testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 9.5: Risk Management Quiz</t>
+  </si>
+  <si>
+    <t>Base Camp: Teamwork Assignment Due</t>
+  </si>
+  <si>
+    <t>Game Dev: Release Your Game</t>
+  </si>
+  <si>
+    <t>AP: Data Collections Due</t>
+  </si>
+  <si>
+    <t>Web Dev: Website Checkpoint 1
+Game Dev: Explore the Industry</t>
+  </si>
+  <si>
+    <t>Web Dev: Website Checkpoint 2</t>
+  </si>
+  <si>
+    <t>AP: Exam Prep</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -513,6 +547,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF555555"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -856,12 +896,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1237,6 +1278,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3048F481-4A4B-498D-A291-01B119D1D7C2}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I277"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1278,7 +1320,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1301,7 +1343,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1324,7 +1366,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1347,7 +1389,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1370,7 +1412,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -1393,7 +1435,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1416,7 +1458,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1439,7 +1481,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1465,7 +1507,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1488,7 +1530,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1514,7 +1556,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1537,7 +1579,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1560,7 +1602,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -1583,7 +1625,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -1606,7 +1648,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -1629,7 +1671,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -1652,7 +1694,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -1675,7 +1717,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -1698,7 +1740,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>9</v>
       </c>
@@ -1721,7 +1763,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -1744,7 +1786,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -1767,7 +1809,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>9</v>
       </c>
@@ -1790,7 +1832,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -1810,7 +1852,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>9</v>
       </c>
@@ -1830,7 +1872,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>9</v>
       </c>
@@ -1850,7 +1892,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>9</v>
       </c>
@@ -1870,7 +1912,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>9</v>
       </c>
@@ -1890,7 +1932,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>9</v>
       </c>
@@ -1910,7 +1952,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>9</v>
       </c>
@@ -1930,7 +1972,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>9</v>
       </c>
@@ -1950,7 +1992,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>9</v>
       </c>
@@ -1973,7 +2015,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>9</v>
       </c>
@@ -1996,7 +2038,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>9</v>
       </c>
@@ -2019,7 +2061,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>9</v>
       </c>
@@ -2042,7 +2084,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>9</v>
       </c>
@@ -2062,7 +2104,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>9</v>
       </c>
@@ -2082,7 +2124,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>9</v>
       </c>
@@ -2102,7 +2144,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>9</v>
       </c>
@@ -2122,7 +2164,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>9</v>
       </c>
@@ -2142,7 +2184,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>9</v>
       </c>
@@ -2162,7 +2204,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>9</v>
       </c>
@@ -2182,7 +2224,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>9</v>
       </c>
@@ -2202,7 +2244,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>9</v>
       </c>
@@ -2222,7 +2264,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>9</v>
       </c>
@@ -2242,7 +2284,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>9</v>
       </c>
@@ -2262,7 +2304,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>9</v>
       </c>
@@ -2282,7 +2324,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>9</v>
       </c>
@@ -2302,7 +2344,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>9</v>
       </c>
@@ -2322,7 +2364,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>9</v>
       </c>
@@ -2342,7 +2384,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>9</v>
       </c>
@@ -2362,7 +2404,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>9</v>
       </c>
@@ -2382,7 +2424,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>9</v>
       </c>
@@ -2402,7 +2444,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>9</v>
       </c>
@@ -2422,7 +2464,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>9</v>
       </c>
@@ -2442,7 +2484,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>9</v>
       </c>
@@ -2462,7 +2504,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>9</v>
       </c>
@@ -2482,7 +2524,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>9</v>
       </c>
@@ -2505,7 +2547,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>9</v>
       </c>
@@ -2528,7 +2570,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>9</v>
       </c>
@@ -2548,7 +2590,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>9</v>
       </c>
@@ -2568,7 +2610,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>9</v>
       </c>
@@ -2588,7 +2630,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>9</v>
       </c>
@@ -2608,7 +2650,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>9</v>
       </c>
@@ -2628,7 +2670,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>9</v>
       </c>
@@ -2648,7 +2690,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>9</v>
       </c>
@@ -2668,7 +2710,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>9</v>
       </c>
@@ -2688,7 +2730,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>9</v>
       </c>
@@ -2708,7 +2750,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>9</v>
       </c>
@@ -2728,7 +2770,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>9</v>
       </c>
@@ -2748,7 +2790,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>9</v>
       </c>
@@ -2771,7 +2813,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>9</v>
       </c>
@@ -2794,7 +2836,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>9</v>
       </c>
@@ -2820,7 +2862,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>9</v>
       </c>
@@ -2843,7 +2885,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>9</v>
       </c>
@@ -2866,7 +2908,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>9</v>
       </c>
@@ -2889,7 +2931,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>9</v>
       </c>
@@ -2912,7 +2954,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>9</v>
       </c>
@@ -2938,7 +2980,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>9</v>
       </c>
@@ -2961,7 +3003,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>9</v>
       </c>
@@ -2987,7 +3029,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>9</v>
       </c>
@@ -3010,7 +3052,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>9</v>
       </c>
@@ -3024,7 +3066,7 @@
         <v>88</v>
       </c>
       <c r="E82" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F82" t="s">
         <v>91</v>
@@ -3033,7 +3075,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>9</v>
       </c>
@@ -3056,7 +3098,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>9</v>
       </c>
@@ -3079,7 +3121,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>9</v>
       </c>
@@ -3102,7 +3144,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>9</v>
       </c>
@@ -3125,7 +3167,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>9</v>
       </c>
@@ -3148,7 +3190,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>9</v>
       </c>
@@ -3171,7 +3213,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>9</v>
       </c>
@@ -3194,7 +3236,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>9</v>
       </c>
@@ -3217,7 +3259,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>9</v>
       </c>
@@ -3240,7 +3282,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>9</v>
       </c>
@@ -3263,7 +3305,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>9</v>
       </c>
@@ -3283,7 +3325,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>9</v>
       </c>
@@ -3294,7 +3336,7 @@
         <v>46119</v>
       </c>
       <c r="D94" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="E94" t="s">
         <v>88</v>
@@ -3303,7 +3345,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>9</v>
       </c>
@@ -3314,7 +3356,7 @@
         <v>46120</v>
       </c>
       <c r="D95" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E95" t="s">
         <v>88</v>
@@ -3323,7 +3365,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>9</v>
       </c>
@@ -3343,7 +3385,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>9</v>
       </c>
@@ -3354,16 +3396,16 @@
         <v>46122</v>
       </c>
       <c r="D97" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="E97" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="H97" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>9</v>
       </c>
@@ -3374,16 +3416,16 @@
         <v>46125</v>
       </c>
       <c r="D98" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E98" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="H98" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>9</v>
       </c>
@@ -3394,16 +3436,16 @@
         <v>46126</v>
       </c>
       <c r="D99" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E99" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H99" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>9</v>
       </c>
@@ -3414,16 +3456,13 @@
         <v>46127</v>
       </c>
       <c r="D100" t="s">
-        <v>98</v>
-      </c>
-      <c r="E100" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H100" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>9</v>
       </c>
@@ -3446,7 +3485,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>9</v>
       </c>
@@ -3457,10 +3496,10 @@
         <v>46129</v>
       </c>
       <c r="D102" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E102" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G102" t="s">
         <v>49</v>
@@ -3469,7 +3508,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>9</v>
       </c>
@@ -3479,9 +3518,6 @@
       <c r="C103" s="1">
         <v>46132</v>
       </c>
-      <c r="D103" t="s">
-        <v>98</v>
-      </c>
       <c r="E103" t="s">
         <v>14</v>
       </c>
@@ -3489,7 +3525,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>9</v>
       </c>
@@ -3499,17 +3535,14 @@
       <c r="C104" s="1">
         <v>46133</v>
       </c>
-      <c r="D104" t="s">
-        <v>98</v>
-      </c>
       <c r="E104" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H104" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>9</v>
       </c>
@@ -3523,13 +3556,13 @@
         <v>38</v>
       </c>
       <c r="E105" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="H105" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>9</v>
       </c>
@@ -3543,13 +3576,13 @@
         <v>38</v>
       </c>
       <c r="E106" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H106" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>9</v>
       </c>
@@ -3560,16 +3593,16 @@
         <v>46136</v>
       </c>
       <c r="D107" t="s">
-        <v>38</v>
+        <v>111</v>
       </c>
       <c r="E107" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="H107" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>9</v>
       </c>
@@ -3582,14 +3615,11 @@
       <c r="D108" t="s">
         <v>38</v>
       </c>
-      <c r="E108" t="s">
-        <v>98</v>
-      </c>
       <c r="H108" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>9</v>
       </c>
@@ -3602,14 +3632,11 @@
       <c r="D109" t="s">
         <v>38</v>
       </c>
-      <c r="E109" t="s">
-        <v>98</v>
-      </c>
       <c r="H109" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>9</v>
       </c>
@@ -3619,14 +3646,14 @@
       <c r="C110" s="1">
         <v>46141</v>
       </c>
-      <c r="E110" t="s">
+      <c r="D110" t="s">
         <v>38</v>
       </c>
       <c r="H110" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>9</v>
       </c>
@@ -3643,7 +3670,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>9</v>
       </c>
@@ -3653,14 +3680,17 @@
       <c r="C112" s="1">
         <v>46143</v>
       </c>
+      <c r="D112" t="s">
+        <v>111</v>
+      </c>
       <c r="E112" t="s">
-        <v>38</v>
+        <v>111</v>
       </c>
       <c r="H112" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>9</v>
       </c>
@@ -3677,7 +3707,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>9</v>
       </c>
@@ -3694,7 +3724,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>9</v>
       </c>
@@ -3704,11 +3734,14 @@
       <c r="C115" s="1">
         <v>46148</v>
       </c>
+      <c r="E115" t="s">
+        <v>38</v>
+      </c>
       <c r="H115" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>9</v>
       </c>
@@ -3718,11 +3751,14 @@
       <c r="C116" s="1">
         <v>46149</v>
       </c>
+      <c r="E116" t="s">
+        <v>38</v>
+      </c>
       <c r="H116" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>9</v>
       </c>
@@ -3732,11 +3768,17 @@
       <c r="C117" s="1">
         <v>46150</v>
       </c>
+      <c r="D117" t="s">
+        <v>111</v>
+      </c>
+      <c r="E117" t="s">
+        <v>111</v>
+      </c>
       <c r="H117" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>9</v>
       </c>
@@ -3750,7 +3792,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>9</v>
       </c>
@@ -3764,7 +3806,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>9</v>
       </c>
@@ -3778,7 +3820,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>9</v>
       </c>
@@ -3792,7 +3834,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>9</v>
       </c>
@@ -3802,11 +3844,17 @@
       <c r="C122" s="1">
         <v>46157</v>
       </c>
+      <c r="D122" t="s">
+        <v>111</v>
+      </c>
+      <c r="E122" t="s">
+        <v>111</v>
+      </c>
       <c r="H122" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>9</v>
       </c>
@@ -3820,7 +3868,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>9</v>
       </c>
@@ -3834,7 +3882,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>9</v>
       </c>
@@ -3848,7 +3896,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>9</v>
       </c>
@@ -3862,7 +3910,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>9</v>
       </c>
@@ -3885,7 +3933,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>9</v>
       </c>
@@ -3908,7 +3956,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>9</v>
       </c>
@@ -3922,7 +3970,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>9</v>
       </c>
@@ -3936,7 +3984,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>9</v>
       </c>
@@ -3950,7 +3998,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>9</v>
       </c>
@@ -3961,10 +4009,10 @@
         <v>46171</v>
       </c>
       <c r="H132" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>9</v>
       </c>
@@ -3978,7 +4026,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>9</v>
       </c>
@@ -3992,7 +4040,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>9</v>
       </c>
@@ -4006,7 +4054,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>9</v>
       </c>
@@ -4020,7 +4068,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>9</v>
       </c>
@@ -4031,10 +4079,10 @@
         <v>46178</v>
       </c>
       <c r="H137" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>9</v>
       </c>
@@ -4048,7 +4096,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>9</v>
       </c>
@@ -4062,16 +4110,19 @@
         <v>15</v>
       </c>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>9</v>
       </c>
       <c r="B140" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C140" s="1">
         <v>46086</v>
       </c>
+      <c r="D140" s="3" t="s">
+        <v>112</v>
+      </c>
       <c r="F140" t="s">
         <v>76</v>
       </c>
@@ -4079,16 +4130,19 @@
         <v>12</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>9</v>
       </c>
       <c r="B141" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C141" s="1">
         <v>46087</v>
       </c>
+      <c r="D141" t="s">
+        <v>113</v>
+      </c>
       <c r="F141" t="s">
         <v>76</v>
       </c>
@@ -4096,16 +4150,19 @@
         <v>12</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>9</v>
       </c>
       <c r="B142" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C142" s="1">
         <v>46090</v>
       </c>
+      <c r="D142" t="s">
+        <v>14</v>
+      </c>
       <c r="F142" t="s">
         <v>76</v>
       </c>
@@ -4113,42 +4170,42 @@
         <v>15</v>
       </c>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>9</v>
       </c>
       <c r="B143" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C143" s="1">
         <v>46091</v>
       </c>
       <c r="D143" t="s">
-        <v>100</v>
-      </c>
-      <c r="E143" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="F143" t="s">
         <v>76</v>
       </c>
       <c r="G143" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H143" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>9</v>
       </c>
       <c r="B144" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C144" s="1">
         <v>46092</v>
       </c>
+      <c r="D144" t="s">
+        <v>86</v>
+      </c>
       <c r="F144" t="s">
         <v>76</v>
       </c>
@@ -4156,16 +4213,19 @@
         <v>15</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>9</v>
       </c>
       <c r="B145" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C145" s="1">
         <v>46093</v>
       </c>
+      <c r="D145" t="s">
+        <v>115</v>
+      </c>
       <c r="F145" t="s">
         <v>76</v>
       </c>
@@ -4173,16 +4233,19 @@
         <v>15</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>9</v>
       </c>
       <c r="B146" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C146" s="1">
         <v>46094</v>
       </c>
+      <c r="D146" t="s">
+        <v>116</v>
+      </c>
       <c r="F146" t="s">
         <v>85</v>
       </c>
@@ -4190,16 +4253,19 @@
         <v>22</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>9</v>
       </c>
       <c r="B147" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C147" s="1">
         <v>46097</v>
       </c>
+      <c r="D147" t="s">
+        <v>117</v>
+      </c>
       <c r="F147" t="s">
         <v>87</v>
       </c>
@@ -4207,16 +4273,19 @@
         <v>25</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>9</v>
       </c>
       <c r="B148" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C148" s="1">
         <v>46098</v>
       </c>
+      <c r="D148" t="s">
+        <v>118</v>
+      </c>
       <c r="F148" t="s">
         <v>87</v>
       </c>
@@ -4224,16 +4293,19 @@
         <v>25</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>9</v>
       </c>
       <c r="B149" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C149" s="1">
         <v>46099</v>
       </c>
+      <c r="D149" t="s">
+        <v>119</v>
+      </c>
       <c r="F149" t="s">
         <v>87</v>
       </c>
@@ -4241,12 +4313,12 @@
         <v>29</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>9</v>
       </c>
       <c r="B150" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C150" s="1">
         <v>46100</v>
@@ -4258,12 +4330,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>9</v>
       </c>
       <c r="B151" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C151" s="1">
         <v>46101</v>
@@ -4275,12 +4347,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>9</v>
       </c>
       <c r="B152" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C152" s="1">
         <v>46104</v>
@@ -4292,12 +4364,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>9</v>
       </c>
       <c r="B153" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C153" s="1">
         <v>46105</v>
@@ -4309,12 +4381,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>9</v>
       </c>
       <c r="B154" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C154" s="1">
         <v>46106</v>
@@ -4326,12 +4398,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>9</v>
       </c>
       <c r="B155" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C155" s="1">
         <v>46107</v>
@@ -4343,30 +4415,39 @@
         <v>15</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>9</v>
       </c>
       <c r="B156" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C156" s="1">
         <v>46108</v>
       </c>
+      <c r="F156" t="s">
+        <v>93</v>
+      </c>
       <c r="H156" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>9</v>
       </c>
       <c r="B157" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C157" s="1">
         <v>46111</v>
       </c>
+      <c r="D157" t="s">
+        <v>35</v>
+      </c>
+      <c r="F157" t="s">
+        <v>35</v>
+      </c>
       <c r="G157" t="s">
         <v>36</v>
       </c>
@@ -4374,16 +4455,22 @@
         <v>37</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>9</v>
       </c>
       <c r="B158" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C158" s="1">
         <v>46112</v>
       </c>
+      <c r="D158" t="s">
+        <v>35</v>
+      </c>
+      <c r="F158" t="s">
+        <v>35</v>
+      </c>
       <c r="G158" t="s">
         <v>36</v>
       </c>
@@ -4391,16 +4478,22 @@
         <v>37</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>9</v>
       </c>
       <c r="B159" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C159" s="1">
         <v>46113</v>
       </c>
+      <c r="D159" t="s">
+        <v>35</v>
+      </c>
+      <c r="F159" t="s">
+        <v>35</v>
+      </c>
       <c r="G159" t="s">
         <v>36</v>
       </c>
@@ -4408,16 +4501,22 @@
         <v>37</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>9</v>
       </c>
       <c r="B160" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C160" s="1">
         <v>46114</v>
       </c>
+      <c r="D160" t="s">
+        <v>35</v>
+      </c>
+      <c r="F160" t="s">
+        <v>35</v>
+      </c>
       <c r="G160" t="s">
         <v>36</v>
       </c>
@@ -4425,16 +4524,22 @@
         <v>37</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>9</v>
       </c>
       <c r="B161" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C161" s="1">
         <v>46115</v>
       </c>
+      <c r="D161" t="s">
+        <v>35</v>
+      </c>
+      <c r="F161" t="s">
+        <v>35</v>
+      </c>
       <c r="G161" t="s">
         <v>36</v>
       </c>
@@ -4442,12 +4547,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>9</v>
       </c>
       <c r="B162" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C162" s="1">
         <v>46118</v>
@@ -4456,12 +4561,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>9</v>
       </c>
       <c r="B163" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C163" s="1">
         <v>46119</v>
@@ -4470,12 +4575,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>9</v>
       </c>
       <c r="B164" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C164" s="1">
         <v>46120</v>
@@ -4484,12 +4589,12 @@
         <v>43</v>
       </c>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>9</v>
       </c>
       <c r="B165" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C165" s="1">
         <v>46121</v>
@@ -4498,12 +4603,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>9</v>
       </c>
       <c r="B166" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C166" s="1">
         <v>46122</v>
@@ -4512,12 +4617,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>9</v>
       </c>
       <c r="B167" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C167" s="1">
         <v>46125</v>
@@ -4526,12 +4631,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>9</v>
       </c>
       <c r="B168" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C168" s="1">
         <v>46126</v>
@@ -4540,12 +4645,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>9</v>
       </c>
       <c r="B169" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C169" s="1">
         <v>46127</v>
@@ -4554,16 +4659,19 @@
         <v>15</v>
       </c>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>9</v>
       </c>
       <c r="B170" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C170" s="1">
         <v>46128</v>
       </c>
+      <c r="D170" t="s">
+        <v>46</v>
+      </c>
       <c r="G170" t="s">
         <v>47</v>
       </c>
@@ -4571,16 +4679,19 @@
         <v>15</v>
       </c>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>9</v>
       </c>
       <c r="B171" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C171" s="1">
         <v>46129</v>
       </c>
+      <c r="D171" t="s">
+        <v>98</v>
+      </c>
       <c r="G171" t="s">
         <v>49</v>
       </c>
@@ -4588,12 +4699,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>9</v>
       </c>
       <c r="B172" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C172" s="1">
         <v>46132</v>
@@ -4602,32 +4713,26 @@
         <v>15</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>9</v>
       </c>
       <c r="B173" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C173" s="1">
         <v>46133</v>
       </c>
-      <c r="E173" t="s">
-        <v>100</v>
-      </c>
-      <c r="G173" t="s">
-        <v>106</v>
-      </c>
       <c r="H173" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>9</v>
       </c>
       <c r="B174" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C174" s="1">
         <v>46134</v>
@@ -4636,12 +4741,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>9</v>
       </c>
       <c r="B175" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C175" s="1">
         <v>46135</v>
@@ -4650,12 +4755,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>9</v>
       </c>
       <c r="B176" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C176" s="1">
         <v>46136</v>
@@ -4664,12 +4769,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>9</v>
       </c>
       <c r="B177" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C177" s="1">
         <v>46139</v>
@@ -4678,12 +4783,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>9</v>
       </c>
       <c r="B178" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C178" s="1">
         <v>46140</v>
@@ -4692,12 +4797,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>9</v>
       </c>
       <c r="B179" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C179" s="1">
         <v>46141</v>
@@ -4706,12 +4811,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>9</v>
       </c>
       <c r="B180" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C180" s="1">
         <v>46142</v>
@@ -4720,26 +4825,26 @@
         <v>15</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>9</v>
       </c>
       <c r="B181" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C181" s="1">
         <v>46143</v>
       </c>
       <c r="H181" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.35">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>9</v>
       </c>
       <c r="B182" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C182" s="1">
         <v>46146</v>
@@ -4748,12 +4853,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>9</v>
       </c>
       <c r="B183" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C183" s="1">
         <v>46147</v>
@@ -4762,12 +4867,12 @@
         <v>63</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>9</v>
       </c>
       <c r="B184" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C184" s="1">
         <v>46148</v>
@@ -4776,12 +4881,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>9</v>
       </c>
       <c r="B185" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C185" s="1">
         <v>46149</v>
@@ -4790,26 +4895,26 @@
         <v>15</v>
       </c>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>9</v>
       </c>
       <c r="B186" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C186" s="1">
         <v>46150</v>
       </c>
       <c r="H186" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.35">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="187" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>9</v>
       </c>
       <c r="B187" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C187" s="1">
         <v>46153</v>
@@ -4818,12 +4923,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>9</v>
       </c>
       <c r="B188" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C188" s="1">
         <v>46154</v>
@@ -4832,12 +4937,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>9</v>
       </c>
       <c r="B189" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C189" s="1">
         <v>46155</v>
@@ -4846,12 +4951,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>9</v>
       </c>
       <c r="B190" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C190" s="1">
         <v>46156</v>
@@ -4860,12 +4965,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>9</v>
       </c>
       <c r="B191" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C191" s="1">
         <v>46157</v>
@@ -4874,12 +4979,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>9</v>
       </c>
       <c r="B192" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C192" s="1">
         <v>46160</v>
@@ -4888,12 +4993,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>9</v>
       </c>
       <c r="B193" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C193" s="1">
         <v>46161</v>
@@ -4902,12 +5007,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>9</v>
       </c>
       <c r="B194" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C194" s="1">
         <v>46162</v>
@@ -4916,12 +5021,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>9</v>
       </c>
       <c r="B195" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C195" s="1">
         <v>46163</v>
@@ -4930,16 +5035,19 @@
         <v>15</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>9</v>
       </c>
       <c r="B196" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C196" s="1">
         <v>46164</v>
       </c>
+      <c r="D196" t="s">
+        <v>46</v>
+      </c>
       <c r="G196" t="s">
         <v>70</v>
       </c>
@@ -4947,16 +5055,19 @@
         <v>15</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>9</v>
       </c>
       <c r="B197" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C197" s="1">
         <v>46167</v>
       </c>
+      <c r="D197" t="s">
+        <v>46</v>
+      </c>
       <c r="G197" t="s">
         <v>71</v>
       </c>
@@ -4964,12 +5075,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>9</v>
       </c>
       <c r="B198" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C198" s="1">
         <v>46168</v>
@@ -4978,12 +5089,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>9</v>
       </c>
       <c r="B199" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C199" s="1">
         <v>46169</v>
@@ -4992,12 +5103,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>9</v>
       </c>
       <c r="B200" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C200" s="1">
         <v>46170</v>
@@ -5006,26 +5117,26 @@
         <v>15</v>
       </c>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>9</v>
       </c>
       <c r="B201" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C201" s="1">
         <v>46171</v>
       </c>
       <c r="H201" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.35">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="202" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>9</v>
       </c>
       <c r="B202" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C202" s="1">
         <v>46174</v>
@@ -5034,12 +5145,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>9</v>
       </c>
       <c r="B203" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C203" s="1">
         <v>46175</v>
@@ -5048,12 +5159,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>9</v>
       </c>
       <c r="B204" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C204" s="1">
         <v>46176</v>
@@ -5062,12 +5173,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>9</v>
       </c>
       <c r="B205" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C205" s="1">
         <v>46177</v>
@@ -5076,26 +5187,26 @@
         <v>15</v>
       </c>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>9</v>
       </c>
       <c r="B206" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C206" s="1">
         <v>46178</v>
       </c>
       <c r="H206" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.35">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="207" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>9</v>
       </c>
       <c r="B207" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C207" s="1">
         <v>46181</v>
@@ -5104,12 +5215,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>9</v>
       </c>
       <c r="B208" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C208" s="1">
         <v>46182</v>
@@ -5123,7 +5234,7 @@
         <v>9</v>
       </c>
       <c r="B209" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C209" s="1">
         <v>46086</v>
@@ -5140,7 +5251,7 @@
         <v>9</v>
       </c>
       <c r="B210" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C210" s="1">
         <v>46087</v>
@@ -5157,11 +5268,14 @@
         <v>9</v>
       </c>
       <c r="B211" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C211" s="1">
         <v>46090</v>
       </c>
+      <c r="D211" t="s">
+        <v>14</v>
+      </c>
       <c r="F211" t="s">
         <v>76</v>
       </c>
@@ -5174,20 +5288,17 @@
         <v>9</v>
       </c>
       <c r="B212" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C212" s="1">
         <v>46091</v>
       </c>
       <c r="D212" t="s">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="F212" t="s">
         <v>76</v>
       </c>
-      <c r="G212" t="s">
-        <v>108</v>
-      </c>
       <c r="H212" t="s">
         <v>17</v>
       </c>
@@ -5197,7 +5308,7 @@
         <v>9</v>
       </c>
       <c r="B213" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C213" s="1">
         <v>46092</v>
@@ -5214,7 +5325,7 @@
         <v>9</v>
       </c>
       <c r="B214" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C214" s="1">
         <v>46093</v>
@@ -5226,27 +5337,24 @@
         <v>15</v>
       </c>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>9</v>
       </c>
       <c r="B215" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C215" s="1">
         <v>46094</v>
       </c>
-      <c r="D215" t="s">
-        <v>109</v>
-      </c>
-      <c r="E215" t="s">
-        <v>109</v>
+      <c r="D215" s="2" t="s">
+        <v>123</v>
       </c>
       <c r="F215" t="s">
         <v>85</v>
       </c>
       <c r="G215" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="H215" t="s">
         <v>22</v>
@@ -5257,7 +5365,7 @@
         <v>9</v>
       </c>
       <c r="B216" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C216" s="1">
         <v>46097</v>
@@ -5274,7 +5382,7 @@
         <v>9</v>
       </c>
       <c r="B217" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C217" s="1">
         <v>46098</v>
@@ -5291,7 +5399,7 @@
         <v>9</v>
       </c>
       <c r="B218" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C218" s="1">
         <v>46099</v>
@@ -5300,7 +5408,7 @@
         <v>87</v>
       </c>
       <c r="G218" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="H218" t="s">
         <v>29</v>
@@ -5311,7 +5419,7 @@
         <v>9</v>
       </c>
       <c r="B219" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C219" s="1">
         <v>46100</v>
@@ -5328,22 +5436,19 @@
         <v>9</v>
       </c>
       <c r="B220" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C220" s="1">
         <v>46101</v>
       </c>
       <c r="D220" t="s">
-        <v>112</v>
-      </c>
-      <c r="E220" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="F220" t="s">
         <v>91</v>
       </c>
       <c r="G220" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H220" t="s">
         <v>25</v>
@@ -5354,7 +5459,7 @@
         <v>9</v>
       </c>
       <c r="B221" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C221" s="1">
         <v>46104</v>
@@ -5368,7 +5473,7 @@
         <v>9</v>
       </c>
       <c r="B222" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C222" s="1">
         <v>46105</v>
@@ -5382,7 +5487,7 @@
         <v>9</v>
       </c>
       <c r="B223" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C223" s="1">
         <v>46106</v>
@@ -5396,7 +5501,7 @@
         <v>9</v>
       </c>
       <c r="B224" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C224" s="1">
         <v>46107</v>
@@ -5410,11 +5515,14 @@
         <v>9</v>
       </c>
       <c r="B225" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C225" s="1">
         <v>46108</v>
       </c>
+      <c r="D225" t="s">
+        <v>124</v>
+      </c>
       <c r="H225" t="s">
         <v>34</v>
       </c>
@@ -5424,11 +5532,17 @@
         <v>9</v>
       </c>
       <c r="B226" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C226" s="1">
         <v>46111</v>
       </c>
+      <c r="D226" t="s">
+        <v>35</v>
+      </c>
+      <c r="F226" t="s">
+        <v>35</v>
+      </c>
       <c r="G226" t="s">
         <v>36</v>
       </c>
@@ -5441,11 +5555,17 @@
         <v>9</v>
       </c>
       <c r="B227" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C227" s="1">
         <v>46112</v>
       </c>
+      <c r="D227" t="s">
+        <v>35</v>
+      </c>
+      <c r="F227" t="s">
+        <v>35</v>
+      </c>
       <c r="G227" t="s">
         <v>36</v>
       </c>
@@ -5458,11 +5578,17 @@
         <v>9</v>
       </c>
       <c r="B228" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C228" s="1">
         <v>46113</v>
       </c>
+      <c r="D228" t="s">
+        <v>35</v>
+      </c>
+      <c r="F228" t="s">
+        <v>35</v>
+      </c>
       <c r="G228" t="s">
         <v>36</v>
       </c>
@@ -5475,11 +5601,17 @@
         <v>9</v>
       </c>
       <c r="B229" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C229" s="1">
         <v>46114</v>
       </c>
+      <c r="D229" t="s">
+        <v>35</v>
+      </c>
+      <c r="F229" t="s">
+        <v>35</v>
+      </c>
       <c r="G229" t="s">
         <v>36</v>
       </c>
@@ -5492,11 +5624,17 @@
         <v>9</v>
       </c>
       <c r="B230" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C230" s="1">
         <v>46115</v>
       </c>
+      <c r="D230" t="s">
+        <v>35</v>
+      </c>
+      <c r="F230" t="s">
+        <v>35</v>
+      </c>
       <c r="G230" t="s">
         <v>36</v>
       </c>
@@ -5509,7 +5647,7 @@
         <v>9</v>
       </c>
       <c r="B231" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C231" s="1">
         <v>46118</v>
@@ -5523,7 +5661,7 @@
         <v>9</v>
       </c>
       <c r="B232" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C232" s="1">
         <v>46119</v>
@@ -5537,7 +5675,7 @@
         <v>9</v>
       </c>
       <c r="B233" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C233" s="1">
         <v>46120</v>
@@ -5551,7 +5689,7 @@
         <v>9</v>
       </c>
       <c r="B234" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C234" s="1">
         <v>46121</v>
@@ -5565,11 +5703,14 @@
         <v>9</v>
       </c>
       <c r="B235" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C235" s="1">
         <v>46122</v>
       </c>
+      <c r="D235" t="s">
+        <v>121</v>
+      </c>
       <c r="H235" t="s">
         <v>15</v>
       </c>
@@ -5579,7 +5720,7 @@
         <v>9</v>
       </c>
       <c r="B236" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C236" s="1">
         <v>46125</v>
@@ -5593,7 +5734,7 @@
         <v>9</v>
       </c>
       <c r="B237" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C237" s="1">
         <v>46126</v>
@@ -5607,7 +5748,7 @@
         <v>9</v>
       </c>
       <c r="B238" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C238" s="1">
         <v>46127</v>
@@ -5621,7 +5762,7 @@
         <v>9</v>
       </c>
       <c r="B239" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C239" s="1">
         <v>46128</v>
@@ -5629,9 +5770,6 @@
       <c r="D239" t="s">
         <v>46</v>
       </c>
-      <c r="E239" t="s">
-        <v>46</v>
-      </c>
       <c r="G239" t="s">
         <v>47</v>
       </c>
@@ -5644,16 +5782,13 @@
         <v>9</v>
       </c>
       <c r="B240" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C240" s="1">
         <v>46129</v>
       </c>
       <c r="D240" t="s">
-        <v>99</v>
-      </c>
-      <c r="E240" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G240" t="s">
         <v>49</v>
@@ -5667,7 +5802,7 @@
         <v>9</v>
       </c>
       <c r="B241" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C241" s="1">
         <v>46132</v>
@@ -5681,7 +5816,7 @@
         <v>9</v>
       </c>
       <c r="B242" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C242" s="1">
         <v>46133</v>
@@ -5695,7 +5830,7 @@
         <v>9</v>
       </c>
       <c r="B243" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C243" s="1">
         <v>46134</v>
@@ -5709,7 +5844,7 @@
         <v>9</v>
       </c>
       <c r="B244" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C244" s="1">
         <v>46135</v>
@@ -5723,11 +5858,14 @@
         <v>9</v>
       </c>
       <c r="B245" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C245" s="1">
         <v>46136</v>
       </c>
+      <c r="D245" t="s">
+        <v>122</v>
+      </c>
       <c r="H245" t="s">
         <v>15</v>
       </c>
@@ -5737,11 +5875,14 @@
         <v>9</v>
       </c>
       <c r="B246" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C246" s="1">
         <v>46139</v>
       </c>
+      <c r="D246" t="s">
+        <v>125</v>
+      </c>
       <c r="H246" t="s">
         <v>15</v>
       </c>
@@ -5751,11 +5892,14 @@
         <v>9</v>
       </c>
       <c r="B247" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C247" s="1">
         <v>46140</v>
       </c>
+      <c r="D247" t="s">
+        <v>125</v>
+      </c>
       <c r="H247" t="s">
         <v>15</v>
       </c>
@@ -5765,11 +5909,14 @@
         <v>9</v>
       </c>
       <c r="B248" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C248" s="1">
         <v>46141</v>
       </c>
+      <c r="D248" t="s">
+        <v>125</v>
+      </c>
       <c r="H248" t="s">
         <v>15</v>
       </c>
@@ -5779,11 +5926,14 @@
         <v>9</v>
       </c>
       <c r="B249" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C249" s="1">
         <v>46142</v>
       </c>
+      <c r="D249" t="s">
+        <v>125</v>
+      </c>
       <c r="H249" t="s">
         <v>15</v>
       </c>
@@ -5793,13 +5943,16 @@
         <v>9</v>
       </c>
       <c r="B250" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C250" s="1">
         <v>46143</v>
       </c>
+      <c r="D250" t="s">
+        <v>125</v>
+      </c>
       <c r="H250" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="251" spans="1:8" x14ac:dyDescent="0.35">
@@ -5807,11 +5960,14 @@
         <v>9</v>
       </c>
       <c r="B251" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C251" s="1">
         <v>46146</v>
       </c>
+      <c r="D251" t="s">
+        <v>125</v>
+      </c>
       <c r="H251" t="s">
         <v>15</v>
       </c>
@@ -5821,11 +5977,14 @@
         <v>9</v>
       </c>
       <c r="B252" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C252" s="1">
         <v>46147</v>
       </c>
+      <c r="D252" t="s">
+        <v>125</v>
+      </c>
       <c r="H252" t="s">
         <v>63</v>
       </c>
@@ -5835,11 +5994,14 @@
         <v>9</v>
       </c>
       <c r="B253" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C253" s="1">
         <v>46148</v>
       </c>
+      <c r="D253" t="s">
+        <v>125</v>
+      </c>
       <c r="H253" t="s">
         <v>15</v>
       </c>
@@ -5849,11 +6011,14 @@
         <v>9</v>
       </c>
       <c r="B254" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C254" s="1">
         <v>46149</v>
       </c>
+      <c r="D254" t="s">
+        <v>125</v>
+      </c>
       <c r="H254" t="s">
         <v>15</v>
       </c>
@@ -5863,13 +6028,16 @@
         <v>9</v>
       </c>
       <c r="B255" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C255" s="1">
         <v>46150</v>
       </c>
+      <c r="D255" t="s">
+        <v>125</v>
+      </c>
       <c r="H255" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="256" spans="1:8" x14ac:dyDescent="0.35">
@@ -5877,11 +6045,14 @@
         <v>9</v>
       </c>
       <c r="B256" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C256" s="1">
         <v>46153</v>
       </c>
+      <c r="D256" t="s">
+        <v>125</v>
+      </c>
       <c r="H256" t="s">
         <v>15</v>
       </c>
@@ -5891,11 +6062,14 @@
         <v>9</v>
       </c>
       <c r="B257" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C257" s="1">
         <v>46154</v>
       </c>
+      <c r="D257" t="s">
+        <v>125</v>
+      </c>
       <c r="H257" t="s">
         <v>15</v>
       </c>
@@ -5905,11 +6079,14 @@
         <v>9</v>
       </c>
       <c r="B258" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C258" s="1">
         <v>46155</v>
       </c>
+      <c r="D258" t="s">
+        <v>125</v>
+      </c>
       <c r="H258" t="s">
         <v>15</v>
       </c>
@@ -5919,7 +6096,7 @@
         <v>9</v>
       </c>
       <c r="B259" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C259" s="1">
         <v>46156</v>
@@ -5933,16 +6110,13 @@
         <v>9</v>
       </c>
       <c r="B260" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C260" s="1">
         <v>46157</v>
       </c>
       <c r="D260" t="s">
-        <v>113</v>
-      </c>
-      <c r="E260" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="H260" t="s">
         <v>15</v>
@@ -5953,7 +6127,7 @@
         <v>9</v>
       </c>
       <c r="B261" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C261" s="1">
         <v>46160</v>
@@ -5967,7 +6141,7 @@
         <v>9</v>
       </c>
       <c r="B262" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C262" s="1">
         <v>46161</v>
@@ -5981,7 +6155,7 @@
         <v>9</v>
       </c>
       <c r="B263" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C263" s="1">
         <v>46162</v>
@@ -5995,7 +6169,7 @@
         <v>9</v>
       </c>
       <c r="B264" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C264" s="1">
         <v>46163</v>
@@ -6009,7 +6183,7 @@
         <v>9</v>
       </c>
       <c r="B265" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C265" s="1">
         <v>46164</v>
@@ -6026,7 +6200,7 @@
         <v>9</v>
       </c>
       <c r="B266" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C266" s="1">
         <v>46167</v>
@@ -6043,7 +6217,7 @@
         <v>9</v>
       </c>
       <c r="B267" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C267" s="1">
         <v>46168</v>
@@ -6057,7 +6231,7 @@
         <v>9</v>
       </c>
       <c r="B268" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C268" s="1">
         <v>46169</v>
@@ -6071,7 +6245,7 @@
         <v>9</v>
       </c>
       <c r="B269" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C269" s="1">
         <v>46170</v>
@@ -6085,13 +6259,13 @@
         <v>9</v>
       </c>
       <c r="B270" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C270" s="1">
         <v>46171</v>
       </c>
       <c r="H270" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="271" spans="1:8" x14ac:dyDescent="0.35">
@@ -6099,7 +6273,7 @@
         <v>9</v>
       </c>
       <c r="B271" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C271" s="1">
         <v>46174</v>
@@ -6113,7 +6287,7 @@
         <v>9</v>
       </c>
       <c r="B272" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C272" s="1">
         <v>46175</v>
@@ -6127,7 +6301,7 @@
         <v>9</v>
       </c>
       <c r="B273" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C273" s="1">
         <v>46176</v>
@@ -6141,7 +6315,7 @@
         <v>9</v>
       </c>
       <c r="B274" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C274" s="1">
         <v>46177</v>
@@ -6155,13 +6329,13 @@
         <v>9</v>
       </c>
       <c r="B275" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C275" s="1">
         <v>46178</v>
       </c>
       <c r="H275" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="276" spans="1:8" x14ac:dyDescent="0.35">
@@ -6169,7 +6343,7 @@
         <v>9</v>
       </c>
       <c r="B276" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C276" s="1">
         <v>46181</v>
@@ -6183,7 +6357,7 @@
         <v>9</v>
       </c>
       <c r="B277" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C277" s="1">
         <v>46182</v>
@@ -6193,7 +6367,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I277" xr:uid="{3048F481-4A4B-498D-A291-01B119D1D7C2}"/>
+  <autoFilter ref="A1:I277" xr:uid="{3048F481-4A4B-498D-A291-01B119D1D7C2}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="AP Computer Science A: Game Design"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>